<commit_message>
Committing both the main and pyqt5UI along with Geo spatial mapping working with right geojson mapping
</commit_message>
<xml_diff>
--- a/Gap Analysis Excels/gap_over_3_months.xlsx
+++ b/Gap Analysis Excels/gap_over_3_months.xlsx
@@ -450,17 +450,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Gap Start Date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Gap End Date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Gap (Days)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Gap Start Date</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Gap End Date</t>
         </is>
       </c>
     </row>
@@ -478,19 +478,19 @@
           <t>Rushey Green</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
+        <v>45385</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>45712</v>
+      </c>
+      <c r="F2" t="n">
         <v>327</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>45385</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>45712</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2185951</v>
+        <v>2348155</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -502,19 +502,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
+        <v>45407</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>45729</v>
+      </c>
+      <c r="F3" t="n">
         <v>322</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>45407</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>45729</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2348155</v>
+        <v>2185951</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -526,14 +526,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
+        <v>45407</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>45729</v>
+      </c>
+      <c r="F4" t="n">
         <v>322</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>45407</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>45729</v>
       </c>
     </row>
     <row r="5">
@@ -550,14 +550,14 @@
           <t>Thamesmead Moorings</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
+        <v>45378</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>45691</v>
+      </c>
+      <c r="F5" t="n">
         <v>313</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>45378</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>45691</v>
       </c>
     </row>
     <row r="6">
@@ -570,14 +570,14 @@
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
+        <v>45393</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>45703</v>
+      </c>
+      <c r="F6" t="n">
         <v>310</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>45393</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>45703</v>
       </c>
     </row>
     <row r="7">
@@ -594,14 +594,14 @@
           <t>Custom House</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>45707</v>
+      </c>
+      <c r="F7" t="n">
         <v>303</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>45404</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>45707</v>
       </c>
     </row>
     <row r="8">
@@ -618,14 +618,14 @@
           <t>Cathall</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>45696</v>
+      </c>
+      <c r="F8" t="n">
         <v>292</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>45404</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>45696</v>
       </c>
     </row>
     <row r="9">
@@ -642,14 +642,14 @@
           <t>Stratford</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
+        <v>45379</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>45670</v>
+      </c>
+      <c r="F9" t="n">
         <v>291</v>
-      </c>
-      <c r="E9" s="2" t="n">
-        <v>45379</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>45670</v>
       </c>
     </row>
     <row r="10">
@@ -666,14 +666,14 @@
           <t>Beckton</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
+        <v>45433</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>45721</v>
+      </c>
+      <c r="F10" t="n">
         <v>288</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>45433</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>45721</v>
       </c>
     </row>
     <row r="11">
@@ -690,14 +690,14 @@
           <t>Green Street East</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
+        <v>45426</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>45713</v>
+      </c>
+      <c r="F11" t="n">
         <v>287</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>45426</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>45713</v>
       </c>
     </row>
     <row r="12">
@@ -714,14 +714,14 @@
           <t>Kidbrooke Park</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
+        <v>45453</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>45733</v>
+      </c>
+      <c r="F12" t="n">
         <v>280</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>45453</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>45733</v>
       </c>
     </row>
     <row r="13">
@@ -738,14 +738,14 @@
           <t>Kidbrooke Park</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
+        <v>45453</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>45730</v>
+      </c>
+      <c r="F13" t="n">
         <v>277</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>45453</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>45730</v>
       </c>
     </row>
     <row r="14">
@@ -762,14 +762,14 @@
           <t>Plaistow North</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="2" t="n">
+        <v>45427</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>45692</v>
+      </c>
+      <c r="F14" t="n">
         <v>265</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>45427</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>45692</v>
       </c>
     </row>
     <row r="15">
@@ -786,14 +786,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="2" t="n">
+        <v>45449</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>45713</v>
+      </c>
+      <c r="F15" t="n">
         <v>264</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>45449</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>45713</v>
       </c>
     </row>
     <row r="16">
@@ -810,14 +810,14 @@
           <t>Charlton Village &amp; Riverside</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" s="2" t="n">
+        <v>45425</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>45681</v>
+      </c>
+      <c r="F16" t="n">
         <v>256</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>45425</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>45681</v>
       </c>
     </row>
     <row r="17">
@@ -834,14 +834,14 @@
           <t>East Ham</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>45698</v>
+      </c>
+      <c r="F17" t="n">
         <v>251</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>45447</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>45698</v>
       </c>
     </row>
     <row r="18">
@@ -858,14 +858,14 @@
           <t>East Ham South</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="2" t="n">
+        <v>45422</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>45666</v>
+      </c>
+      <c r="F18" t="n">
         <v>244</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>45422</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>45666</v>
       </c>
     </row>
     <row r="19">
@@ -882,67 +882,67 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="2" t="n">
+        <v>45435</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>45673</v>
+      </c>
+      <c r="F19" t="n">
         <v>238</v>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>45435</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>45673</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2971912</v>
+        <v>3189473</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+          <t>East Ham</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>45397</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>45628</v>
+      </c>
+      <c r="F20" t="n">
         <v>231</v>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>45442</v>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>45673</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3189473</v>
+        <v>2971912</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>East Ham</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>45442</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>45673</v>
+      </c>
+      <c r="F21" t="n">
         <v>231</v>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>45397</v>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>45628</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1810843</v>
+        <v>3219822</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -951,22 +951,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
+          <t>Green Street East</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>45419</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>45643</v>
+      </c>
+      <c r="F22" t="n">
         <v>224</v>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>45475</v>
-      </c>
-      <c r="F22" s="2" t="n">
-        <v>45699</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3219822</v>
+        <v>1810843</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -975,17 +975,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Green Street East</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>45699</v>
+      </c>
+      <c r="F23" t="n">
         <v>224</v>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>45419</v>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>45643</v>
       </c>
     </row>
     <row r="24">
@@ -1002,14 +1002,14 @@
           <t>Boleyn</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="2" t="n">
+        <v>45499</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>45714</v>
+      </c>
+      <c r="F24" t="n">
         <v>215</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>45499</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>45714</v>
       </c>
     </row>
     <row r="25">
@@ -1026,14 +1026,14 @@
           <t>Northbury</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" s="2" t="n">
+        <v>45408</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>45619</v>
+      </c>
+      <c r="F25" t="n">
         <v>211</v>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>45408</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>45619</v>
       </c>
     </row>
     <row r="26">
@@ -1050,14 +1050,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" s="2" t="n">
+        <v>45462</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>45672</v>
+      </c>
+      <c r="F26" t="n">
         <v>210</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>45462</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>45672</v>
       </c>
     </row>
     <row r="27">
@@ -1074,14 +1074,14 @@
           <t>Beckton</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" s="2" t="n">
+        <v>45481</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>45690</v>
+      </c>
+      <c r="F27" t="n">
         <v>209</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>45481</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>45690</v>
       </c>
     </row>
     <row r="28">
@@ -1098,14 +1098,14 @@
           <t>Manor Park</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" s="2" t="n">
+        <v>45406</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>45614</v>
+      </c>
+      <c r="F28" t="n">
         <v>208</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>45406</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>45614</v>
       </c>
     </row>
     <row r="29">
@@ -1122,14 +1122,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="2" t="n">
+        <v>45490</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>45695</v>
+      </c>
+      <c r="F29" t="n">
         <v>205</v>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>45490</v>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>45695</v>
       </c>
     </row>
     <row r="30">
@@ -1146,14 +1146,14 @@
           <t>Thamesmead Moorings</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" s="2" t="n">
+        <v>45478</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>45680</v>
+      </c>
+      <c r="F30" t="n">
         <v>202</v>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>45478</v>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>45680</v>
       </c>
     </row>
     <row r="31">
@@ -1170,14 +1170,14 @@
           <t>Plaistow South</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D31" s="2" t="n">
+        <v>45464</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>45664</v>
+      </c>
+      <c r="F31" t="n">
         <v>200</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>45464</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>45664</v>
       </c>
     </row>
     <row r="32">
@@ -1194,14 +1194,14 @@
           <t>Bethnal Green West</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="2" t="n">
+        <v>45502</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>45699</v>
+      </c>
+      <c r="F32" t="n">
         <v>197</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>45502</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>45699</v>
       </c>
     </row>
     <row r="33">
@@ -1218,14 +1218,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="2" t="n">
+        <v>45441</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>45636</v>
+      </c>
+      <c r="F33" t="n">
         <v>195</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>45441</v>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>45636</v>
       </c>
     </row>
     <row r="34">
@@ -1242,14 +1242,14 @@
           <t>Plaistow South</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" s="2" t="n">
+        <v>45407</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>45601</v>
+      </c>
+      <c r="F34" t="n">
         <v>194</v>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>45407</v>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>45601</v>
       </c>
     </row>
     <row r="35">
@@ -1266,19 +1266,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="2" t="n">
+        <v>45446</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>45637</v>
+      </c>
+      <c r="F35" t="n">
         <v>191</v>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>45446</v>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>45637</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3088350</v>
+        <v>3247141</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1287,22 +1287,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Lea Bridge</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
+          <t>East Ham</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>45664</v>
+      </c>
+      <c r="F36" t="n">
         <v>189</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>45545</v>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>45734</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3247141</v>
+        <v>3088350</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1311,22 +1311,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>East Ham</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
+          <t>Lea Bridge</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="n">
+        <v>45545</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>45734</v>
+      </c>
+      <c r="F37" t="n">
         <v>189</v>
-      </c>
-      <c r="E37" s="2" t="n">
-        <v>45475</v>
-      </c>
-      <c r="F37" s="2" t="n">
-        <v>45664</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1366008</v>
+        <v>3312013</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1335,22 +1335,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Stockwell West &amp; Larkhall</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
+          <t>East Ham South</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>45502</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>45686</v>
+      </c>
+      <c r="F38" t="n">
         <v>184</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>45512</v>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>45696</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>3312013</v>
+        <v>1366008</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1359,22 +1359,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>East Ham South</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
+          <t>Stockwell West &amp; Larkhall</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>45512</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>45696</v>
+      </c>
+      <c r="F39" t="n">
         <v>184</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>45502</v>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>45686</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>2592091</v>
+        <v>2762903</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -1383,22 +1383,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Royal Victoria</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
+          <t>Green Street East</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>45433</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>45615</v>
+      </c>
+      <c r="F40" t="n">
         <v>182</v>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>45632</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>2762903</v>
+        <v>2941628</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1407,66 +1407,66 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Green Street East</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
+          <t>Belvedere</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="n">
+        <v>45499</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>45681</v>
+      </c>
+      <c r="F41" t="n">
         <v>182</v>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>45433</v>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>45615</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>2941628</v>
+        <v>3003762</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Belvedere</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" s="2" t="n">
+        <v>45397</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>45579</v>
+      </c>
+      <c r="F42" t="n">
         <v>182</v>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>45499</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>45681</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>3003762</v>
+        <v>3229982</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="n">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Plaistow South</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>45454</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>45636</v>
+      </c>
+      <c r="F43" t="n">
         <v>182</v>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>45397</v>
-      </c>
-      <c r="F43" s="2" t="n">
-        <v>45579</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>3229982</v>
+        <v>2592091</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1475,22 +1475,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Plaistow South</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
+          <t>Royal Victoria</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>45632</v>
+      </c>
+      <c r="F44" t="n">
         <v>182</v>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>45454</v>
-      </c>
-      <c r="F44" s="2" t="n">
-        <v>45636</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>2873515</v>
+        <v>3189476</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
@@ -1499,22 +1499,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mile End</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
+          <t>East Ham South</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>45448</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>45628</v>
+      </c>
+      <c r="F45" t="n">
         <v>180</v>
-      </c>
-      <c r="E45" s="2" t="n">
-        <v>45533</v>
-      </c>
-      <c r="F45" s="2" t="n">
-        <v>45713</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>3189476</v>
+        <v>2873515</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1523,17 +1523,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>East Ham South</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
+          <t>Mile End</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>45533</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>45713</v>
+      </c>
+      <c r="F46" t="n">
         <v>180</v>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>45448</v>
-      </c>
-      <c r="F46" s="2" t="n">
-        <v>45628</v>
       </c>
     </row>
     <row r="47">
@@ -1550,62 +1550,62 @@
           <t>Custom House</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D47" s="2" t="n">
+        <v>45512</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>45691</v>
+      </c>
+      <c r="F47" t="n">
         <v>179</v>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>45512</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>45691</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3085505</v>
+        <v>3174557</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Royal Victoria</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
+          <t>Stratford</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>45376</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>45554</v>
+      </c>
+      <c r="F48" t="n">
         <v>178</v>
-      </c>
-      <c r="E48" s="2" t="n">
-        <v>45373</v>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>45551</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3174557</v>
+        <v>3085505</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Stratford</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
+          <t>Royal Victoria</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>45373</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>45551</v>
+      </c>
+      <c r="F49" t="n">
         <v>178</v>
-      </c>
-      <c r="E49" s="2" t="n">
-        <v>45376</v>
-      </c>
-      <c r="F49" s="2" t="n">
-        <v>45554</v>
       </c>
     </row>
     <row r="50">
@@ -1622,19 +1622,19 @@
           <t>Stratford</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D50" s="2" t="n">
+        <v>45428</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>45604</v>
+      </c>
+      <c r="F50" t="n">
         <v>176</v>
-      </c>
-      <c r="E50" s="2" t="n">
-        <v>45428</v>
-      </c>
-      <c r="F50" s="2" t="n">
-        <v>45604</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2327403</v>
+        <v>3127237</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1643,17 +1643,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Custom House</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="n">
+        <v>45453</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>45628</v>
+      </c>
+      <c r="F51" t="n">
         <v>175</v>
-      </c>
-      <c r="E51" s="2" t="n">
-        <v>45414</v>
-      </c>
-      <c r="F51" s="2" t="n">
-        <v>45589</v>
       </c>
     </row>
     <row r="52">
@@ -1670,19 +1670,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="D52" s="2" t="n">
+        <v>45534</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>45709</v>
+      </c>
+      <c r="F52" t="n">
         <v>175</v>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>45534</v>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>45709</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>3127237</v>
+        <v>2327403</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1691,85 +1691,85 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
+          <t>Custom House</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>45414</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>45589</v>
+      </c>
+      <c r="F53" t="n">
         <v>175</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>45453</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>45628</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>1823758</v>
+        <v>3223524</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="n">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Beckton</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>45464</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>45632</v>
+      </c>
+      <c r="F54" t="n">
         <v>168</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>45524</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>45692</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2180279</v>
+        <v>1823758</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Brownswood</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" s="2" t="n">
+        <v>45524</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>45692</v>
+      </c>
+      <c r="F55" t="n">
         <v>168</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>45386</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>45554</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>3223524</v>
+        <v>2180279</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Beckton</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
+          <t>Brownswood</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>45386</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>45554</v>
+      </c>
+      <c r="F56" t="n">
         <v>168</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>45464</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>45632</v>
       </c>
     </row>
     <row r="57">
@@ -1786,14 +1786,14 @@
           <t>East Ham South</t>
         </is>
       </c>
-      <c r="D57" t="n">
+      <c r="D57" s="2" t="n">
+        <v>45467</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>45630</v>
+      </c>
+      <c r="F57" t="n">
         <v>163</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>45467</v>
-      </c>
-      <c r="F57" s="2" t="n">
-        <v>45630</v>
       </c>
     </row>
     <row r="58">
@@ -1810,14 +1810,14 @@
           <t>Cathall</t>
         </is>
       </c>
-      <c r="D58" t="n">
+      <c r="D58" s="2" t="n">
+        <v>45433</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>45595</v>
+      </c>
+      <c r="F58" t="n">
         <v>162</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>45433</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>45595</v>
       </c>
     </row>
     <row r="59">
@@ -1834,34 +1834,38 @@
           <t>Hainault</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D59" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>45636</v>
+      </c>
+      <c r="F59" t="n">
         <v>161</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>45475</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>45636</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>668464</v>
+        <v>2680677</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Not provided</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="n">
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>New Cross Gate</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>45393</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>45553</v>
+      </c>
+      <c r="F60" t="n">
         <v>160</v>
-      </c>
-      <c r="E60" s="2" t="n">
-        <v>45434</v>
-      </c>
-      <c r="F60" s="2" t="n">
-        <v>45594</v>
       </c>
     </row>
     <row r="61">
@@ -1878,38 +1882,34 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D61" t="n">
+      <c r="D61" s="2" t="n">
+        <v>45527</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>45687</v>
+      </c>
+      <c r="F61" t="n">
         <v>160</v>
-      </c>
-      <c r="E61" s="2" t="n">
-        <v>45527</v>
-      </c>
-      <c r="F61" s="2" t="n">
-        <v>45687</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>2680677</v>
+        <v>668464</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>New Cross Gate</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
+          <t>Not provided</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>45594</v>
+      </c>
+      <c r="F62" t="n">
         <v>160</v>
-      </c>
-      <c r="E62" s="2" t="n">
-        <v>45393</v>
-      </c>
-      <c r="F62" s="2" t="n">
-        <v>45553</v>
       </c>
     </row>
     <row r="63">
@@ -1926,14 +1926,14 @@
           <t>Seven Kings</t>
         </is>
       </c>
-      <c r="D63" t="n">
+      <c r="D63" s="2" t="n">
+        <v>45447</v>
+      </c>
+      <c r="E63" s="2" t="n">
+        <v>45603</v>
+      </c>
+      <c r="F63" t="n">
         <v>156</v>
-      </c>
-      <c r="E63" s="2" t="n">
-        <v>45447</v>
-      </c>
-      <c r="F63" s="2" t="n">
-        <v>45603</v>
       </c>
     </row>
     <row r="64">
@@ -1950,14 +1950,14 @@
           <t>Shadwell</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D64" s="2" t="n">
+        <v>45413</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>45569</v>
+      </c>
+      <c r="F64" t="n">
         <v>156</v>
-      </c>
-      <c r="E64" s="2" t="n">
-        <v>45413</v>
-      </c>
-      <c r="F64" s="2" t="n">
-        <v>45569</v>
       </c>
     </row>
     <row r="65">
@@ -1970,19 +1970,19 @@
         </is>
       </c>
       <c r="C65" t="inlineStr"/>
-      <c r="D65" t="n">
+      <c r="D65" s="2" t="n">
+        <v>45405</v>
+      </c>
+      <c r="E65" s="2" t="n">
+        <v>45559</v>
+      </c>
+      <c r="F65" t="n">
         <v>154</v>
-      </c>
-      <c r="E65" s="2" t="n">
-        <v>45405</v>
-      </c>
-      <c r="F65" s="2" t="n">
-        <v>45559</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>2342833</v>
+        <v>3169623</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1994,23 +1994,23 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D66" t="n">
+      <c r="D66" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>45604</v>
+      </c>
+      <c r="F66" t="n">
         <v>154</v>
-      </c>
-      <c r="E66" s="2" t="n">
-        <v>45484</v>
-      </c>
-      <c r="F66" s="2" t="n">
-        <v>45638</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>2974767</v>
+        <v>2342833</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2018,71 +2018,71 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D67" t="n">
+      <c r="D67" s="2" t="n">
+        <v>45484</v>
+      </c>
+      <c r="E67" s="2" t="n">
+        <v>45638</v>
+      </c>
+      <c r="F67" t="n">
         <v>154</v>
-      </c>
-      <c r="E67" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>45604</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>2987509</v>
+        <v>3020451</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D68" t="n">
+          <t>South Bermondsey</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>45471</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>45625</v>
+      </c>
+      <c r="F68" t="n">
         <v>154</v>
-      </c>
-      <c r="E68" s="2" t="n">
-        <v>45419</v>
-      </c>
-      <c r="F68" s="2" t="n">
-        <v>45573</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>3020451</v>
+        <v>2974767</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>South Bermondsey</t>
-        </is>
-      </c>
-      <c r="D69" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E69" s="2" t="n">
+        <v>45604</v>
+      </c>
+      <c r="F69" t="n">
         <v>154</v>
-      </c>
-      <c r="E69" s="2" t="n">
-        <v>45471</v>
-      </c>
-      <c r="F69" s="2" t="n">
-        <v>45625</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>3169623</v>
+        <v>2987509</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2090,19 +2090,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D70" t="n">
+      <c r="D70" s="2" t="n">
+        <v>45419</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>45573</v>
+      </c>
+      <c r="F70" t="n">
         <v>154</v>
-      </c>
-      <c r="E70" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F70" s="2" t="n">
-        <v>45604</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2201710</v>
+        <v>3254889</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -2111,22 +2111,22 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Boleyn</t>
-        </is>
-      </c>
-      <c r="D71" t="n">
+          <t>Beckton</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>45561</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>45713</v>
+      </c>
+      <c r="F71" t="n">
         <v>152</v>
-      </c>
-      <c r="E71" s="2" t="n">
-        <v>45532</v>
-      </c>
-      <c r="F71" s="2" t="n">
-        <v>45684</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>3254889</v>
+        <v>2201710</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -2135,17 +2135,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Beckton</t>
-        </is>
-      </c>
-      <c r="D72" t="n">
+          <t>Boleyn</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>45532</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>45684</v>
+      </c>
+      <c r="F72" t="n">
         <v>152</v>
-      </c>
-      <c r="E72" s="2" t="n">
-        <v>45561</v>
-      </c>
-      <c r="F72" s="2" t="n">
-        <v>45713</v>
       </c>
     </row>
     <row r="73">
@@ -2162,19 +2162,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D73" t="n">
+      <c r="D73" s="2" t="n">
+        <v>45572</v>
+      </c>
+      <c r="E73" s="2" t="n">
+        <v>45723</v>
+      </c>
+      <c r="F73" t="n">
         <v>151</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>45572</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>45723</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>2887461</v>
+        <v>3168211</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2183,22 +2183,22 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Royal Victoria</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
+          <t>Bethnal Green East</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>45562</v>
+      </c>
+      <c r="F74" t="n">
         <v>150</v>
-      </c>
-      <c r="E74" s="2" t="n">
-        <v>45524</v>
-      </c>
-      <c r="F74" s="2" t="n">
-        <v>45674</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>3168211</v>
+        <v>2887461</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2207,17 +2207,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Bethnal Green East</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
+          <t>Royal Victoria</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>45524</v>
+      </c>
+      <c r="E75" s="2" t="n">
+        <v>45674</v>
+      </c>
+      <c r="F75" t="n">
         <v>150</v>
-      </c>
-      <c r="E75" s="2" t="n">
-        <v>45412</v>
-      </c>
-      <c r="F75" s="2" t="n">
-        <v>45562</v>
       </c>
     </row>
     <row r="76">
@@ -2234,14 +2234,14 @@
           <t>Grove Green</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D76" s="2" t="n">
+        <v>45540</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>45687</v>
+      </c>
+      <c r="F76" t="n">
         <v>147</v>
-      </c>
-      <c r="E76" s="2" t="n">
-        <v>45540</v>
-      </c>
-      <c r="F76" s="2" t="n">
-        <v>45687</v>
       </c>
     </row>
     <row r="77">
@@ -2258,14 +2258,14 @@
           <t>Canning Town South</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D77" s="2" t="n">
+        <v>45428</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>45575</v>
+      </c>
+      <c r="F77" t="n">
         <v>147</v>
-      </c>
-      <c r="E77" s="2" t="n">
-        <v>45428</v>
-      </c>
-      <c r="F77" s="2" t="n">
-        <v>45575</v>
       </c>
     </row>
     <row r="78">
@@ -2282,14 +2282,14 @@
           <t>East Ham</t>
         </is>
       </c>
-      <c r="D78" t="n">
+      <c r="D78" s="2" t="n">
+        <v>45470</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>45617</v>
+      </c>
+      <c r="F78" t="n">
         <v>147</v>
-      </c>
-      <c r="E78" s="2" t="n">
-        <v>45470</v>
-      </c>
-      <c r="F78" s="2" t="n">
-        <v>45617</v>
       </c>
     </row>
     <row r="79">
@@ -2306,14 +2306,14 @@
           <t>Beam Park</t>
         </is>
       </c>
-      <c r="D79" t="n">
+      <c r="D79" s="2" t="n">
+        <v>45586</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>45733</v>
+      </c>
+      <c r="F79" t="n">
         <v>147</v>
-      </c>
-      <c r="E79" s="2" t="n">
-        <v>45586</v>
-      </c>
-      <c r="F79" s="2" t="n">
-        <v>45733</v>
       </c>
     </row>
     <row r="80">
@@ -2330,14 +2330,14 @@
           <t>Little Ilford</t>
         </is>
       </c>
-      <c r="D80" t="n">
+      <c r="D80" s="2" t="n">
+        <v>45443</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>45589</v>
+      </c>
+      <c r="F80" t="n">
         <v>146</v>
-      </c>
-      <c r="E80" s="2" t="n">
-        <v>45443</v>
-      </c>
-      <c r="F80" s="2" t="n">
-        <v>45589</v>
       </c>
     </row>
     <row r="81">
@@ -2354,19 +2354,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D81" t="n">
+      <c r="D81" s="2" t="n">
+        <v>45492</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>45636</v>
+      </c>
+      <c r="F81" t="n">
         <v>144</v>
-      </c>
-      <c r="E81" s="2" t="n">
-        <v>45492</v>
-      </c>
-      <c r="F81" s="2" t="n">
-        <v>45636</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>2836031</v>
+        <v>2883270</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2375,22 +2375,22 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Custom House</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>45559</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>45702</v>
+      </c>
+      <c r="F82" t="n">
         <v>143</v>
-      </c>
-      <c r="E82" s="2" t="n">
-        <v>45397</v>
-      </c>
-      <c r="F82" s="2" t="n">
-        <v>45540</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>2883270</v>
+        <v>2836031</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2399,17 +2399,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
+          <t>Custom House</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>45397</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>45540</v>
+      </c>
+      <c r="F83" t="n">
         <v>143</v>
-      </c>
-      <c r="E83" s="2" t="n">
-        <v>45559</v>
-      </c>
-      <c r="F83" s="2" t="n">
-        <v>45702</v>
       </c>
     </row>
     <row r="84">
@@ -2426,14 +2426,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D84" t="n">
+      <c r="D84" s="2" t="n">
+        <v>45404</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>45546</v>
+      </c>
+      <c r="F84" t="n">
         <v>142</v>
-      </c>
-      <c r="E84" s="2" t="n">
-        <v>45404</v>
-      </c>
-      <c r="F84" s="2" t="n">
-        <v>45546</v>
       </c>
     </row>
     <row r="85">
@@ -2450,14 +2450,14 @@
           <t>Royal Victoria</t>
         </is>
       </c>
-      <c r="D85" t="n">
+      <c r="D85" s="2" t="n">
+        <v>45475</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>45615</v>
+      </c>
+      <c r="F85" t="n">
         <v>140</v>
-      </c>
-      <c r="E85" s="2" t="n">
-        <v>45475</v>
-      </c>
-      <c r="F85" s="2" t="n">
-        <v>45615</v>
       </c>
     </row>
     <row r="86">
@@ -2474,19 +2474,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D86" t="n">
+      <c r="D86" s="2" t="n">
+        <v>45433</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>45573</v>
+      </c>
+      <c r="F86" t="n">
         <v>140</v>
-      </c>
-      <c r="E86" s="2" t="n">
-        <v>45433</v>
-      </c>
-      <c r="F86" s="2" t="n">
-        <v>45573</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>3222145</v>
+        <v>3222155</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
@@ -2495,22 +2495,22 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Green Street West</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
+          <t>Cann Hall</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>45456</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>45596</v>
+      </c>
+      <c r="F87" t="n">
         <v>140</v>
-      </c>
-      <c r="E87" s="2" t="n">
-        <v>45456</v>
-      </c>
-      <c r="F87" s="2" t="n">
-        <v>45596</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>3222155</v>
+        <v>3222145</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2519,17 +2519,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Cann Hall</t>
-        </is>
-      </c>
-      <c r="D88" t="n">
+          <t>Green Street West</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>45456</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>45596</v>
+      </c>
+      <c r="F88" t="n">
         <v>140</v>
-      </c>
-      <c r="E88" s="2" t="n">
-        <v>45456</v>
-      </c>
-      <c r="F88" s="2" t="n">
-        <v>45596</v>
       </c>
     </row>
     <row r="89">
@@ -2546,14 +2546,14 @@
           <t>Canning Town South</t>
         </is>
       </c>
-      <c r="D89" t="n">
+      <c r="D89" s="2" t="n">
+        <v>45497</v>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>45637</v>
+      </c>
+      <c r="F89" t="n">
         <v>140</v>
-      </c>
-      <c r="E89" s="2" t="n">
-        <v>45497</v>
-      </c>
-      <c r="F89" s="2" t="n">
-        <v>45637</v>
       </c>
     </row>
     <row r="90">
@@ -2570,14 +2570,14 @@
           <t>East Ham South</t>
         </is>
       </c>
-      <c r="D90" t="n">
+      <c r="D90" s="2" t="n">
+        <v>45421</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>45560</v>
+      </c>
+      <c r="F90" t="n">
         <v>139</v>
-      </c>
-      <c r="E90" s="2" t="n">
-        <v>45421</v>
-      </c>
-      <c r="F90" s="2" t="n">
-        <v>45560</v>
       </c>
     </row>
     <row r="91">
@@ -2594,67 +2594,67 @@
           <t>Green Street West</t>
         </is>
       </c>
-      <c r="D91" t="n">
+      <c r="D91" s="2" t="n">
+        <v>45540</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>45678</v>
+      </c>
+      <c r="F91" t="n">
         <v>138</v>
-      </c>
-      <c r="E91" s="2" t="n">
-        <v>45540</v>
-      </c>
-      <c r="F91" s="2" t="n">
-        <v>45678</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>361217</v>
+        <v>3075195</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Custom House</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
+          <t>Canning Town South</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>45558</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>45695</v>
+      </c>
+      <c r="F92" t="n">
         <v>137</v>
-      </c>
-      <c r="E92" s="2" t="n">
-        <v>45541</v>
-      </c>
-      <c r="F92" s="2" t="n">
-        <v>45678</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>3075195</v>
+        <v>361217</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Canning Town South</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
+          <t>Custom House</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="n">
+        <v>45541</v>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>45678</v>
+      </c>
+      <c r="F93" t="n">
         <v>137</v>
-      </c>
-      <c r="E93" s="2" t="n">
-        <v>45558</v>
-      </c>
-      <c r="F93" s="2" t="n">
-        <v>45695</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>2797604</v>
+        <v>3022841</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -2663,22 +2663,22 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Canning Town North</t>
-        </is>
-      </c>
-      <c r="D94" t="n">
+          <t>Whitechapel</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="n">
+        <v>45545</v>
+      </c>
+      <c r="E94" s="2" t="n">
+        <v>45681</v>
+      </c>
+      <c r="F94" t="n">
         <v>136</v>
-      </c>
-      <c r="E94" s="2" t="n">
-        <v>45412</v>
-      </c>
-      <c r="F94" s="2" t="n">
-        <v>45548</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>3022841</v>
+        <v>2797604</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -2687,17 +2687,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whitechapel</t>
-        </is>
-      </c>
-      <c r="D95" t="n">
+          <t>Canning Town North</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="n">
+        <v>45412</v>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>45548</v>
+      </c>
+      <c r="F95" t="n">
         <v>136</v>
-      </c>
-      <c r="E95" s="2" t="n">
-        <v>45545</v>
-      </c>
-      <c r="F95" s="2" t="n">
-        <v>45681</v>
       </c>
     </row>
     <row r="96">
@@ -2714,14 +2714,14 @@
           <t>Wall End</t>
         </is>
       </c>
-      <c r="D96" t="n">
+      <c r="D96" s="2" t="n">
+        <v>45569</v>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>45703</v>
+      </c>
+      <c r="F96" t="n">
         <v>134</v>
-      </c>
-      <c r="E96" s="2" t="n">
-        <v>45569</v>
-      </c>
-      <c r="F96" s="2" t="n">
-        <v>45703</v>
       </c>
     </row>
     <row r="97">
@@ -2738,19 +2738,19 @@
           <t>Victoria</t>
         </is>
       </c>
-      <c r="D97" t="n">
+      <c r="D97" s="2" t="n">
+        <v>45414</v>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>45548</v>
+      </c>
+      <c r="F97" t="n">
         <v>134</v>
-      </c>
-      <c r="E97" s="2" t="n">
-        <v>45414</v>
-      </c>
-      <c r="F97" s="2" t="n">
-        <v>45548</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>2464236</v>
+        <v>3226051</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -2759,22 +2759,22 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Stratford Olympic Park</t>
-        </is>
-      </c>
-      <c r="D98" t="n">
+          <t>Plaistow West &amp; Canning Town East</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="n">
+        <v>45554</v>
+      </c>
+      <c r="E98" s="2" t="n">
+        <v>45687</v>
+      </c>
+      <c r="F98" t="n">
         <v>133</v>
-      </c>
-      <c r="E98" s="2" t="n">
-        <v>45399</v>
-      </c>
-      <c r="F98" s="2" t="n">
-        <v>45532</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>3226051</v>
+        <v>2464236</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -2783,17 +2783,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Plaistow West &amp; Canning Town East</t>
-        </is>
-      </c>
-      <c r="D99" t="n">
+          <t>Stratford Olympic Park</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="n">
+        <v>45399</v>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>45532</v>
+      </c>
+      <c r="F99" t="n">
         <v>133</v>
-      </c>
-      <c r="E99" s="2" t="n">
-        <v>45554</v>
-      </c>
-      <c r="F99" s="2" t="n">
-        <v>45687</v>
       </c>
     </row>
     <row r="100">
@@ -2810,14 +2810,14 @@
           <t>Plaistow North</t>
         </is>
       </c>
-      <c r="D100" t="n">
+      <c r="D100" s="2" t="n">
+        <v>45406</v>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>45538</v>
+      </c>
+      <c r="F100" t="n">
         <v>132</v>
-      </c>
-      <c r="E100" s="2" t="n">
-        <v>45406</v>
-      </c>
-      <c r="F100" s="2" t="n">
-        <v>45538</v>
       </c>
     </row>
     <row r="101">
@@ -2834,67 +2834,67 @@
           <t>East Ham South</t>
         </is>
       </c>
-      <c r="D101" t="n">
+      <c r="D101" s="2" t="n">
+        <v>45426</v>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>45555</v>
+      </c>
+      <c r="F101" t="n">
         <v>129</v>
-      </c>
-      <c r="E101" s="2" t="n">
-        <v>45426</v>
-      </c>
-      <c r="F101" s="2" t="n">
-        <v>45555</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>3004459</v>
+        <v>3184479</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>East Ham South</t>
-        </is>
-      </c>
-      <c r="D102" t="n">
+          <t>Stratford Olympic Park</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="n">
+        <v>45414</v>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>45541</v>
+      </c>
+      <c r="F102" t="n">
         <v>127</v>
-      </c>
-      <c r="E102" s="2" t="n">
-        <v>45489</v>
-      </c>
-      <c r="F102" s="2" t="n">
-        <v>45616</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>3184479</v>
+        <v>3004459</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Stratford Olympic Park</t>
-        </is>
-      </c>
-      <c r="D103" t="n">
+          <t>East Ham South</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="n">
+        <v>45489</v>
+      </c>
+      <c r="E103" s="2" t="n">
+        <v>45616</v>
+      </c>
+      <c r="F103" t="n">
         <v>127</v>
-      </c>
-      <c r="E103" s="2" t="n">
-        <v>45414</v>
-      </c>
-      <c r="F103" s="2" t="n">
-        <v>45541</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>359492</v>
+        <v>1640496</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -2903,46 +2903,46 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D104" t="n">
+          <t>Beckton</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E104" s="2" t="n">
+        <v>45560</v>
+      </c>
+      <c r="F104" t="n">
         <v>126</v>
-      </c>
-      <c r="E104" s="2" t="n">
-        <v>45422</v>
-      </c>
-      <c r="F104" s="2" t="n">
-        <v>45548</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1640496</v>
+        <v>2101882</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Beckton</t>
-        </is>
-      </c>
-      <c r="D105" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="n">
+        <v>45552</v>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>45678</v>
+      </c>
+      <c r="F105" t="n">
         <v>126</v>
-      </c>
-      <c r="E105" s="2" t="n">
-        <v>45434</v>
-      </c>
-      <c r="F105" s="2" t="n">
-        <v>45560</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>2101882</v>
+        <v>2403384</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -2951,41 +2951,41 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D106" t="n">
+          <t>Plaistow South</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="n">
+        <v>45601</v>
+      </c>
+      <c r="E106" s="2" t="n">
+        <v>45727</v>
+      </c>
+      <c r="F106" t="n">
         <v>126</v>
-      </c>
-      <c r="E106" s="2" t="n">
-        <v>45552</v>
-      </c>
-      <c r="F106" s="2" t="n">
-        <v>45678</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>2403384</v>
+        <v>359492</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Plaistow South</t>
-        </is>
-      </c>
-      <c r="D107" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="n">
+        <v>45422</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>45548</v>
+      </c>
+      <c r="F107" t="n">
         <v>126</v>
-      </c>
-      <c r="E107" s="2" t="n">
-        <v>45601</v>
-      </c>
-      <c r="F107" s="2" t="n">
-        <v>45727</v>
       </c>
     </row>
     <row r="108">
@@ -3002,19 +3002,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D108" t="n">
+      <c r="D108" s="2" t="n">
+        <v>45413</v>
+      </c>
+      <c r="E108" s="2" t="n">
+        <v>45537</v>
+      </c>
+      <c r="F108" t="n">
         <v>124</v>
-      </c>
-      <c r="E108" s="2" t="n">
-        <v>45413</v>
-      </c>
-      <c r="F108" s="2" t="n">
-        <v>45537</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>2419075</v>
+        <v>3234149</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -3023,22 +3023,22 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D109" t="n">
+          <t>East Ham</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="n">
+        <v>45520</v>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>45643</v>
+      </c>
+      <c r="F109" t="n">
         <v>123</v>
-      </c>
-      <c r="E109" s="2" t="n">
-        <v>45456</v>
-      </c>
-      <c r="F109" s="2" t="n">
-        <v>45579</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>3234149</v>
+        <v>2419075</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -3047,17 +3047,17 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>East Ham</t>
-        </is>
-      </c>
-      <c r="D110" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="n">
+        <v>45456</v>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>45579</v>
+      </c>
+      <c r="F110" t="n">
         <v>123</v>
-      </c>
-      <c r="E110" s="2" t="n">
-        <v>45520</v>
-      </c>
-      <c r="F110" s="2" t="n">
-        <v>45643</v>
       </c>
     </row>
     <row r="111">
@@ -3074,14 +3074,14 @@
           <t>Beckton</t>
         </is>
       </c>
-      <c r="D111" t="n">
+      <c r="D111" s="2" t="n">
+        <v>45544</v>
+      </c>
+      <c r="E111" s="2" t="n">
+        <v>45665</v>
+      </c>
+      <c r="F111" t="n">
         <v>121</v>
-      </c>
-      <c r="E111" s="2" t="n">
-        <v>45544</v>
-      </c>
-      <c r="F111" s="2" t="n">
-        <v>45665</v>
       </c>
     </row>
     <row r="112">
@@ -3098,14 +3098,14 @@
           <t>Stratford</t>
         </is>
       </c>
-      <c r="D112" t="n">
+      <c r="D112" s="2" t="n">
+        <v>45566</v>
+      </c>
+      <c r="E112" s="2" t="n">
+        <v>45686</v>
+      </c>
+      <c r="F112" t="n">
         <v>120</v>
-      </c>
-      <c r="E112" s="2" t="n">
-        <v>45566</v>
-      </c>
-      <c r="F112" s="2" t="n">
-        <v>45686</v>
       </c>
     </row>
     <row r="113">
@@ -3122,14 +3122,14 @@
           <t>Leytonstone</t>
         </is>
       </c>
-      <c r="D113" t="n">
+      <c r="D113" s="2" t="n">
+        <v>45470</v>
+      </c>
+      <c r="E113" s="2" t="n">
+        <v>45589</v>
+      </c>
+      <c r="F113" t="n">
         <v>119</v>
-      </c>
-      <c r="E113" s="2" t="n">
-        <v>45470</v>
-      </c>
-      <c r="F113" s="2" t="n">
-        <v>45589</v>
       </c>
     </row>
     <row r="114">
@@ -3146,14 +3146,14 @@
           <t>Beckton</t>
         </is>
       </c>
-      <c r="D114" t="n">
+      <c r="D114" s="2" t="n">
+        <v>45558</v>
+      </c>
+      <c r="E114" s="2" t="n">
+        <v>45677</v>
+      </c>
+      <c r="F114" t="n">
         <v>119</v>
-      </c>
-      <c r="E114" s="2" t="n">
-        <v>45558</v>
-      </c>
-      <c r="F114" s="2" t="n">
-        <v>45677</v>
       </c>
     </row>
     <row r="115">
@@ -3170,14 +3170,14 @@
           <t>Loughton Roding</t>
         </is>
       </c>
-      <c r="D115" t="n">
+      <c r="D115" s="2" t="n">
+        <v>45473</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>45589</v>
+      </c>
+      <c r="F115" t="n">
         <v>116</v>
-      </c>
-      <c r="E115" s="2" t="n">
-        <v>45473</v>
-      </c>
-      <c r="F115" s="2" t="n">
-        <v>45589</v>
       </c>
     </row>
     <row r="116">
@@ -3194,14 +3194,14 @@
           <t>St. Giles</t>
         </is>
       </c>
-      <c r="D116" t="n">
+      <c r="D116" s="2" t="n">
+        <v>45490</v>
+      </c>
+      <c r="E116" s="2" t="n">
+        <v>45604</v>
+      </c>
+      <c r="F116" t="n">
         <v>114</v>
-      </c>
-      <c r="E116" s="2" t="n">
-        <v>45490</v>
-      </c>
-      <c r="F116" s="2" t="n">
-        <v>45604</v>
       </c>
     </row>
     <row r="117">
@@ -3218,14 +3218,14 @@
           <t>Little Ilford</t>
         </is>
       </c>
-      <c r="D117" t="n">
+      <c r="D117" s="2" t="n">
+        <v>45434</v>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>45547</v>
+      </c>
+      <c r="F117" t="n">
         <v>113</v>
-      </c>
-      <c r="E117" s="2" t="n">
-        <v>45434</v>
-      </c>
-      <c r="F117" s="2" t="n">
-        <v>45547</v>
       </c>
     </row>
     <row r="118">
@@ -3242,14 +3242,14 @@
           <t>Royal Victoria</t>
         </is>
       </c>
-      <c r="D118" t="n">
+      <c r="D118" s="2" t="n">
+        <v>45442</v>
+      </c>
+      <c r="E118" s="2" t="n">
+        <v>45554</v>
+      </c>
+      <c r="F118" t="n">
         <v>112</v>
-      </c>
-      <c r="E118" s="2" t="n">
-        <v>45442</v>
-      </c>
-      <c r="F118" s="2" t="n">
-        <v>45554</v>
       </c>
     </row>
     <row r="119">
@@ -3266,19 +3266,19 @@
           <t>Stratford Olympic Park</t>
         </is>
       </c>
-      <c r="D119" t="n">
+      <c r="D119" s="2" t="n">
+        <v>45554</v>
+      </c>
+      <c r="E119" s="2" t="n">
+        <v>45666</v>
+      </c>
+      <c r="F119" t="n">
         <v>112</v>
-      </c>
-      <c r="E119" s="2" t="n">
-        <v>45554</v>
-      </c>
-      <c r="F119" s="2" t="n">
-        <v>45666</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>3251635</v>
+        <v>3303632</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -3287,22 +3287,22 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Valentines</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
+          <t>Custom House</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="n">
+        <v>45517</v>
+      </c>
+      <c r="E120" s="2" t="n">
+        <v>45629</v>
+      </c>
+      <c r="F120" t="n">
         <v>112</v>
-      </c>
-      <c r="E120" s="2" t="n">
-        <v>45453</v>
-      </c>
-      <c r="F120" s="2" t="n">
-        <v>45565</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>3303632</v>
+        <v>3251635</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -3311,17 +3311,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Custom House</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
+          <t>Valentines</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="n">
+        <v>45453</v>
+      </c>
+      <c r="E121" s="2" t="n">
+        <v>45565</v>
+      </c>
+      <c r="F121" t="n">
         <v>112</v>
-      </c>
-      <c r="E121" s="2" t="n">
-        <v>45517</v>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>45629</v>
       </c>
     </row>
     <row r="122">
@@ -3338,14 +3338,14 @@
           <t>Woolwich Arsenal</t>
         </is>
       </c>
-      <c r="D122" t="n">
+      <c r="D122" s="2" t="n">
+        <v>45483</v>
+      </c>
+      <c r="E122" s="2" t="n">
+        <v>45594</v>
+      </c>
+      <c r="F122" t="n">
         <v>111</v>
-      </c>
-      <c r="E122" s="2" t="n">
-        <v>45483</v>
-      </c>
-      <c r="F122" s="2" t="n">
-        <v>45594</v>
       </c>
     </row>
     <row r="123">
@@ -3362,14 +3362,14 @@
           <t>Canning Town South</t>
         </is>
       </c>
-      <c r="D123" t="n">
+      <c r="D123" s="2" t="n">
+        <v>45441</v>
+      </c>
+      <c r="E123" s="2" t="n">
+        <v>45552</v>
+      </c>
+      <c r="F123" t="n">
         <v>111</v>
-      </c>
-      <c r="E123" s="2" t="n">
-        <v>45441</v>
-      </c>
-      <c r="F123" s="2" t="n">
-        <v>45552</v>
       </c>
     </row>
     <row r="124">
@@ -3386,19 +3386,19 @@
           <t>Whitechapel</t>
         </is>
       </c>
-      <c r="D124" t="n">
+      <c r="D124" s="2" t="n">
+        <v>45490</v>
+      </c>
+      <c r="E124" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="F124" t="n">
         <v>110</v>
-      </c>
-      <c r="E124" s="2" t="n">
-        <v>45490</v>
-      </c>
-      <c r="F124" s="2" t="n">
-        <v>45600</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>2836031</v>
+        <v>3099168</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -3407,17 +3407,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Custom House</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
+          <t>West Ham</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="n">
+        <v>45374</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>45483</v>
+      </c>
+      <c r="F125" t="n">
         <v>109</v>
-      </c>
-      <c r="E125" s="2" t="n">
-        <v>45569</v>
-      </c>
-      <c r="F125" s="2" t="n">
-        <v>45678</v>
       </c>
     </row>
     <row r="126">
@@ -3434,19 +3434,19 @@
           <t>Beckton</t>
         </is>
       </c>
-      <c r="D126" t="n">
+      <c r="D126" s="2" t="n">
+        <v>45460</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>45569</v>
+      </c>
+      <c r="F126" t="n">
         <v>109</v>
-      </c>
-      <c r="E126" s="2" t="n">
-        <v>45460</v>
-      </c>
-      <c r="F126" s="2" t="n">
-        <v>45569</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>3099168</v>
+        <v>2836031</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -3455,17 +3455,17 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>West Ham</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
+          <t>Custom House</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>45569</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>45678</v>
+      </c>
+      <c r="F127" t="n">
         <v>109</v>
-      </c>
-      <c r="E127" s="2" t="n">
-        <v>45374</v>
-      </c>
-      <c r="F127" s="2" t="n">
-        <v>45483</v>
       </c>
     </row>
     <row r="128">
@@ -3482,19 +3482,19 @@
           <t>Custom House</t>
         </is>
       </c>
-      <c r="D128" t="n">
+      <c r="D128" s="2" t="n">
+        <v>45481</v>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>45588</v>
+      </c>
+      <c r="F128" t="n">
         <v>107</v>
-      </c>
-      <c r="E128" s="2" t="n">
-        <v>45481</v>
-      </c>
-      <c r="F128" s="2" t="n">
-        <v>45588</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>2747586</v>
+        <v>2832026</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -3503,22 +3503,22 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Plumstead &amp; Glyndon</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
+          <t>Custom House</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="n">
+        <v>45593</v>
+      </c>
+      <c r="E129" s="2" t="n">
+        <v>45699</v>
+      </c>
+      <c r="F129" t="n">
         <v>106</v>
-      </c>
-      <c r="E129" s="2" t="n">
-        <v>45596</v>
-      </c>
-      <c r="F129" s="2" t="n">
-        <v>45702</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>2832026</v>
+        <v>2747586</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -3527,17 +3527,17 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Custom House</t>
-        </is>
-      </c>
-      <c r="D130" t="n">
+          <t>Plumstead &amp; Glyndon</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>45596</v>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>45702</v>
+      </c>
+      <c r="F130" t="n">
         <v>106</v>
-      </c>
-      <c r="E130" s="2" t="n">
-        <v>45593</v>
-      </c>
-      <c r="F130" s="2" t="n">
-        <v>45699</v>
       </c>
     </row>
     <row r="131">
@@ -3554,14 +3554,14 @@
           <t>Canning Town South</t>
         </is>
       </c>
-      <c r="D131" t="n">
+      <c r="D131" s="2" t="n">
+        <v>45441</v>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>45547</v>
+      </c>
+      <c r="F131" t="n">
         <v>106</v>
-      </c>
-      <c r="E131" s="2" t="n">
-        <v>45441</v>
-      </c>
-      <c r="F131" s="2" t="n">
-        <v>45547</v>
       </c>
     </row>
     <row r="132">
@@ -3578,43 +3578,43 @@
           <t>Beckton</t>
         </is>
       </c>
-      <c r="D132" t="n">
+      <c r="D132" s="2" t="n">
+        <v>45567</v>
+      </c>
+      <c r="E132" s="2" t="n">
+        <v>45672</v>
+      </c>
+      <c r="F132" t="n">
         <v>105</v>
-      </c>
-      <c r="E132" s="2" t="n">
-        <v>45567</v>
-      </c>
-      <c r="F132" s="2" t="n">
-        <v>45672</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>1841973</v>
+        <v>1981377</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Green Street East</t>
-        </is>
-      </c>
-      <c r="D133" t="n">
+          <t>Plaistow North</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="n">
+        <v>45512</v>
+      </c>
+      <c r="E133" s="2" t="n">
+        <v>45615</v>
+      </c>
+      <c r="F133" t="n">
         <v>103</v>
-      </c>
-      <c r="E133" s="2" t="n">
-        <v>45527</v>
-      </c>
-      <c r="F133" s="2" t="n">
-        <v>45630</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>1981377</v>
+        <v>3090166</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -3623,46 +3623,46 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Plaistow North</t>
-        </is>
-      </c>
-      <c r="D134" t="n">
+          <t>West Ham</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="n">
+        <v>45512</v>
+      </c>
+      <c r="E134" s="2" t="n">
+        <v>45615</v>
+      </c>
+      <c r="F134" t="n">
         <v>103</v>
-      </c>
-      <c r="E134" s="2" t="n">
-        <v>45512</v>
-      </c>
-      <c r="F134" s="2" t="n">
-        <v>45615</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>3090166</v>
+        <v>3341997</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>West Ham</t>
-        </is>
-      </c>
-      <c r="D135" t="n">
+          <t>Beckton</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="n">
+        <v>45539</v>
+      </c>
+      <c r="E135" s="2" t="n">
+        <v>45642</v>
+      </c>
+      <c r="F135" t="n">
         <v>103</v>
-      </c>
-      <c r="E135" s="2" t="n">
-        <v>45512</v>
-      </c>
-      <c r="F135" s="2" t="n">
-        <v>45615</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>3341997</v>
+        <v>1841973</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -3671,17 +3671,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Beckton</t>
-        </is>
-      </c>
-      <c r="D136" t="n">
+          <t>Green Street East</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="n">
+        <v>45527</v>
+      </c>
+      <c r="E136" s="2" t="n">
+        <v>45630</v>
+      </c>
+      <c r="F136" t="n">
         <v>103</v>
-      </c>
-      <c r="E136" s="2" t="n">
-        <v>45539</v>
-      </c>
-      <c r="F136" s="2" t="n">
-        <v>45642</v>
       </c>
     </row>
     <row r="137">
@@ -3694,14 +3694,14 @@
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
-      <c r="D137" t="n">
+      <c r="D137" s="2" t="n">
+        <v>45594</v>
+      </c>
+      <c r="E137" s="2" t="n">
+        <v>45696</v>
+      </c>
+      <c r="F137" t="n">
         <v>102</v>
-      </c>
-      <c r="E137" s="2" t="n">
-        <v>45594</v>
-      </c>
-      <c r="F137" s="2" t="n">
-        <v>45696</v>
       </c>
     </row>
     <row r="138">
@@ -3718,14 +3718,14 @@
           <t>Canning Town South</t>
         </is>
       </c>
-      <c r="D138" t="n">
+      <c r="D138" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E138" s="2" t="n">
+        <v>45552</v>
+      </c>
+      <c r="F138" t="n">
         <v>102</v>
-      </c>
-      <c r="E138" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F138" s="2" t="n">
-        <v>45552</v>
       </c>
     </row>
     <row r="139">
@@ -3742,14 +3742,14 @@
           <t>Custom House</t>
         </is>
       </c>
-      <c r="D139" t="n">
+      <c r="D139" s="2" t="n">
+        <v>45534</v>
+      </c>
+      <c r="E139" s="2" t="n">
+        <v>45635</v>
+      </c>
+      <c r="F139" t="n">
         <v>101</v>
-      </c>
-      <c r="E139" s="2" t="n">
-        <v>45534</v>
-      </c>
-      <c r="F139" s="2" t="n">
-        <v>45635</v>
       </c>
     </row>
     <row r="140">
@@ -3766,19 +3766,19 @@
           <t>Canning Town North</t>
         </is>
       </c>
-      <c r="D140" t="n">
+      <c r="D140" s="2" t="n">
+        <v>45497</v>
+      </c>
+      <c r="E140" s="2" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F140" t="n">
         <v>100</v>
-      </c>
-      <c r="E140" s="2" t="n">
-        <v>45497</v>
-      </c>
-      <c r="F140" s="2" t="n">
-        <v>45597</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>2567179</v>
+        <v>3292384</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -3787,17 +3787,17 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D141" t="n">
+          <t>East Wickham</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="n">
+        <v>45491</v>
+      </c>
+      <c r="E141" s="2" t="n">
+        <v>45589</v>
+      </c>
+      <c r="F141" t="n">
         <v>98</v>
-      </c>
-      <c r="E141" s="2" t="n">
-        <v>45474</v>
-      </c>
-      <c r="F141" s="2" t="n">
-        <v>45572</v>
       </c>
     </row>
     <row r="142">
@@ -3814,19 +3814,19 @@
           <t>Blackfen &amp; Lamorbey</t>
         </is>
       </c>
-      <c r="D142" t="n">
+      <c r="D142" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E142" s="2" t="n">
+        <v>45548</v>
+      </c>
+      <c r="F142" t="n">
         <v>98</v>
-      </c>
-      <c r="E142" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F142" s="2" t="n">
-        <v>45548</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>3292384</v>
+        <v>3396830</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -3835,22 +3835,22 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>East Wickham</t>
-        </is>
-      </c>
-      <c r="D143" t="n">
+          <t>Woolwich Arsenal</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>45607</v>
+      </c>
+      <c r="E143" s="2" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F143" t="n">
         <v>98</v>
-      </c>
-      <c r="E143" s="2" t="n">
-        <v>45491</v>
-      </c>
-      <c r="F143" s="2" t="n">
-        <v>45589</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>3396830</v>
+        <v>3400389</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -3859,22 +3859,22 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Woolwich Arsenal</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
+          <t>Plumstead &amp; Glyndon</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="n">
+        <v>45607</v>
+      </c>
+      <c r="E144" s="2" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F144" t="n">
         <v>98</v>
-      </c>
-      <c r="E144" s="2" t="n">
-        <v>45607</v>
-      </c>
-      <c r="F144" s="2" t="n">
-        <v>45705</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>3400389</v>
+        <v>2567179</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -3883,22 +3883,22 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Plumstead &amp; Glyndon</t>
-        </is>
-      </c>
-      <c r="D145" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="E145" s="2" t="n">
+        <v>45572</v>
+      </c>
+      <c r="F145" t="n">
         <v>98</v>
-      </c>
-      <c r="E145" s="2" t="n">
-        <v>45607</v>
-      </c>
-      <c r="F145" s="2" t="n">
-        <v>45705</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>3112553</v>
+        <v>3329933</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -3907,65 +3907,65 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Canning Town South</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="n">
+        <v>45582</v>
+      </c>
+      <c r="E146" s="2" t="n">
+        <v>45679</v>
+      </c>
+      <c r="F146" t="n">
         <v>97</v>
-      </c>
-      <c r="E146" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F146" s="2" t="n">
-        <v>45547</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>3292384</v>
+        <v>3112553</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>East Wickham</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
+          <t>Canning Town South</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E147" s="2" t="n">
+        <v>45547</v>
+      </c>
+      <c r="F147" t="n">
         <v>97</v>
-      </c>
-      <c r="E147" s="2" t="n">
-        <v>45610</v>
-      </c>
-      <c r="F147" s="2" t="n">
-        <v>45707</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>3329933</v>
+        <v>3292384</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
+          <t>East Wickham</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="n">
+        <v>45610</v>
+      </c>
+      <c r="E148" s="2" t="n">
+        <v>45707</v>
+      </c>
+      <c r="F148" t="n">
         <v>97</v>
-      </c>
-      <c r="E148" s="2" t="n">
-        <v>45582</v>
-      </c>
-      <c r="F148" s="2" t="n">
-        <v>45679</v>
       </c>
     </row>
     <row r="149">
@@ -3982,14 +3982,14 @@
           <t>East Ham</t>
         </is>
       </c>
-      <c r="D149" t="n">
+      <c r="D149" s="2" t="n">
+        <v>45373</v>
+      </c>
+      <c r="E149" s="2" t="n">
+        <v>45469</v>
+      </c>
+      <c r="F149" t="n">
         <v>96</v>
-      </c>
-      <c r="E149" s="2" t="n">
-        <v>45373</v>
-      </c>
-      <c r="F149" s="2" t="n">
-        <v>45469</v>
       </c>
     </row>
     <row r="150">
@@ -4006,14 +4006,14 @@
           <t>Boleyn</t>
         </is>
       </c>
-      <c r="D150" t="n">
+      <c r="D150" s="2" t="n">
+        <v>45450</v>
+      </c>
+      <c r="E150" s="2" t="n">
+        <v>45545</v>
+      </c>
+      <c r="F150" t="n">
         <v>95</v>
-      </c>
-      <c r="E150" s="2" t="n">
-        <v>45450</v>
-      </c>
-      <c r="F150" s="2" t="n">
-        <v>45545</v>
       </c>
     </row>
     <row r="151">
@@ -4030,19 +4030,19 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D151" t="n">
+      <c r="D151" s="2" t="n">
+        <v>45495</v>
+      </c>
+      <c r="E151" s="2" t="n">
+        <v>45589</v>
+      </c>
+      <c r="F151" t="n">
         <v>94</v>
-      </c>
-      <c r="E151" s="2" t="n">
-        <v>45495</v>
-      </c>
-      <c r="F151" s="2" t="n">
-        <v>45589</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>2250774</v>
+        <v>3143622</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -4051,22 +4051,22 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Loughton Roding</t>
-        </is>
-      </c>
-      <c r="D152" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>45461</v>
+      </c>
+      <c r="E152" s="2" t="n">
+        <v>45555</v>
+      </c>
+      <c r="F152" t="n">
         <v>94</v>
-      </c>
-      <c r="E152" s="2" t="n">
-        <v>45379</v>
-      </c>
-      <c r="F152" s="2" t="n">
-        <v>45473</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>3143622</v>
+        <v>3355052</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D153" t="n">
+          <t>Bow West</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="n">
+        <v>45545</v>
+      </c>
+      <c r="E153" s="2" t="n">
+        <v>45639</v>
+      </c>
+      <c r="F153" t="n">
         <v>94</v>
-      </c>
-      <c r="E153" s="2" t="n">
-        <v>45461</v>
-      </c>
-      <c r="F153" s="2" t="n">
-        <v>45555</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>3355052</v>
+        <v>2250774</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -4099,41 +4099,41 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Bow West</t>
-        </is>
-      </c>
-      <c r="D154" t="n">
+          <t>Loughton Roding</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="n">
+        <v>45379</v>
+      </c>
+      <c r="E154" s="2" t="n">
+        <v>45473</v>
+      </c>
+      <c r="F154" t="n">
         <v>94</v>
-      </c>
-      <c r="E154" s="2" t="n">
-        <v>45545</v>
-      </c>
-      <c r="F154" s="2" t="n">
-        <v>45639</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>359335</v>
+        <v>2212093</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Village</t>
-        </is>
-      </c>
-      <c r="D155" t="n">
+          <t>Royal Albert</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="n">
+        <v>45638</v>
+      </c>
+      <c r="E155" s="2" t="n">
+        <v>45729</v>
+      </c>
+      <c r="F155" t="n">
         <v>91</v>
-      </c>
-      <c r="E155" s="2" t="n">
-        <v>45621</v>
-      </c>
-      <c r="F155" s="2" t="n">
-        <v>45712</v>
       </c>
     </row>
     <row r="156">
@@ -4146,38 +4146,38 @@
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
-      <c r="D156" t="n">
+      <c r="D156" s="2" t="n">
+        <v>45502</v>
+      </c>
+      <c r="E156" s="2" t="n">
+        <v>45593</v>
+      </c>
+      <c r="F156" t="n">
         <v>91</v>
-      </c>
-      <c r="E156" s="2" t="n">
-        <v>45502</v>
-      </c>
-      <c r="F156" s="2" t="n">
-        <v>45593</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>2212093</v>
+        <v>359335</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Royal Albert</t>
-        </is>
-      </c>
-      <c r="D157" t="n">
+          <t>Village</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>45621</v>
+      </c>
+      <c r="E157" s="2" t="n">
+        <v>45712</v>
+      </c>
+      <c r="F157" t="n">
         <v>91</v>
-      </c>
-      <c r="E157" s="2" t="n">
-        <v>45638</v>
-      </c>
-      <c r="F157" s="2" t="n">
-        <v>45729</v>
       </c>
     </row>
     <row r="158">
@@ -4194,62 +4194,62 @@
           <t>Green Street East</t>
         </is>
       </c>
-      <c r="D158" t="n">
+      <c r="D158" s="2" t="n">
+        <v>45636</v>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>45727</v>
+      </c>
+      <c r="F158" t="n">
         <v>91</v>
-      </c>
-      <c r="E158" s="2" t="n">
-        <v>45636</v>
-      </c>
-      <c r="F158" s="2" t="n">
-        <v>45727</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>3250185</v>
+        <v>3280768</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Boleyn</t>
-        </is>
-      </c>
-      <c r="D159" t="n">
+          <t>East Ham South</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="n">
+        <v>45490</v>
+      </c>
+      <c r="E159" s="2" t="n">
+        <v>45581</v>
+      </c>
+      <c r="F159" t="n">
         <v>91</v>
-      </c>
-      <c r="E159" s="2" t="n">
-        <v>45534</v>
-      </c>
-      <c r="F159" s="2" t="n">
-        <v>45625</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>3280768</v>
+        <v>3250185</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>East Ham South</t>
-        </is>
-      </c>
-      <c r="D160" t="n">
+          <t>Boleyn</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="n">
+        <v>45534</v>
+      </c>
+      <c r="E160" s="2" t="n">
+        <v>45625</v>
+      </c>
+      <c r="F160" t="n">
         <v>91</v>
-      </c>
-      <c r="E160" s="2" t="n">
-        <v>45490</v>
-      </c>
-      <c r="F160" s="2" t="n">
-        <v>45581</v>
       </c>
     </row>
     <row r="161">
@@ -4266,14 +4266,14 @@
           <t>Royal Albert</t>
         </is>
       </c>
-      <c r="D161" t="n">
+      <c r="D161" s="2" t="n">
+        <v>45583</v>
+      </c>
+      <c r="E161" s="2" t="n">
+        <v>45674</v>
+      </c>
+      <c r="F161" t="n">
         <v>91</v>
-      </c>
-      <c r="E161" s="2" t="n">
-        <v>45583</v>
-      </c>
-      <c r="F161" s="2" t="n">
-        <v>45674</v>
       </c>
     </row>
     <row r="162">
@@ -4290,14 +4290,14 @@
           <t>East Ham South</t>
         </is>
       </c>
-      <c r="D162" t="n">
+      <c r="D162" s="2" t="n">
+        <v>45645</v>
+      </c>
+      <c r="E162" s="2" t="n">
+        <v>45736</v>
+      </c>
+      <c r="F162" t="n">
         <v>91</v>
-      </c>
-      <c r="E162" s="2" t="n">
-        <v>45645</v>
-      </c>
-      <c r="F162" s="2" t="n">
-        <v>45736</v>
       </c>
     </row>
   </sheetData>

</xml_diff>